<commit_message>
test(corpus): add genuine 1904 and scanned encrypted PDF fixtures
</commit_message>
<xml_diff>
--- a/corpus/xlsx/workbook-1904-note.xlsx
+++ b/corpus/xlsx/workbook-1904-note.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="true"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -248,7 +248,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>1462</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -256,7 +256,7 @@
         <v>1462</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>2924</v>
+        <v>1462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(corpus): rebuild the Office and PDF corpus with stable LibreOffice 24.2
Regenerate the 34 DOCX, XLSX, PPTX, ODT, ODS, ODP and PDF fixtures with a
stable LibreOffice release, record reproducibility (timestamps and
tool-generated IDs only), list every file's requirement in the README,
and run the build script's tests in verify.
</commit_message>
<xml_diff>
--- a/corpus/xlsx/workbook-1904-note.xlsx
+++ b/corpus/xlsx/workbook-1904-note.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="true"/>
   <workbookProtection/>
   <bookViews>
@@ -129,37 +129,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -233,7 +233,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -264,8 +264,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>